<commit_message>
Added Priority and Edit functionality
</commit_message>
<xml_diff>
--- a/vehicle_list.xlsx
+++ b/vehicle_list.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -406,6 +406,9 @@
       <c r="B1" t="str">
         <v>isAccepted</v>
       </c>
+      <c r="C1" t="str">
+        <v>Priority</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -414,18 +417,35 @@
       <c r="B2" t="b">
         <v>1</v>
       </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>XYZ-123</v>
+        <v>XYZ-1234</v>
       </c>
       <c r="B3" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>BOGRA-123</v>
+      </c>
+      <c r="B4" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>